<commit_message>
Q1.22 em formato de tabela
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/semana1_diagnostico.xlsx
+++ b/kobo/semana1_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2510,17 +2510,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>q1_22_nota</t>
+          <t>t1_22</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Q1.22. Para cada elemento selecionado, qual sua relação com a escola/comunidade? Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
+          <t>Q1.22. Para cada elemento selecionado, qual sua relação com a escola/comunidade?</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -2530,7 +2530,11 @@
           <t>${q1_21} != ''</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>table-list</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
@@ -2548,7 +2552,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Rios/córregos</t>
+          <t>Rios/córregos</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -2576,7 +2580,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Lagoas/lagos/reservatórios</t>
+          <t>Lagoas/lagos/reservatórios</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -2604,7 +2608,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Vegetação</t>
+          <t>Vegetação</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -2632,7 +2636,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Parques</t>
+          <t>Parques</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -2660,7 +2664,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Encostas</t>
+          <t>Encostas</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -2688,7 +2692,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Agricultura</t>
+          <t>Agricultura</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -2716,7 +2720,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Indústria</t>
+          <t>Indústria</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
@@ -2744,7 +2748,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Mineração</t>
+          <t>Mineração</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
@@ -2772,7 +2776,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Aterro/lixão</t>
+          <t>Aterro/lixão</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -2800,7 +2804,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Áreas queimadas</t>
+          <t>Áreas queimadas</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -2828,7 +2832,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Áreas inundáveis</t>
+          <t>Áreas inundáveis</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -2856,7 +2860,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Áreas degradadas</t>
+          <t>Áreas degradadas</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -2884,7 +2888,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Q1.22 — Relação: Outros</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -2902,19 +2906,11 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>select_multiple ativ_econ</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>q1_23</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Q1.23. Principais atividades econômicas do território</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
@@ -2926,24 +2922,24 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>q1_23_outro</t>
+          <t>q1_22_nota</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Nota para tutoria: um mesmo elemento pode ter mais de uma relação ao mesmo tempo (ex.: um rio pode ser, simultaneamente, ambiente e cultura, ou risco e uso comunitário) — marque quantas se aplicarem.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>selected(${q1_23}, 'outro')</t>
+          <t>${q1_21} != ''</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -2954,17 +2950,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple ativ_econ</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>q1_24</t>
+          <t>q1_23</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade?</t>
+          <t>Q1.23. Principais atividades econômicas do território</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -2983,26 +2979,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>q1_25</t>
+          <t>q1_23_outro</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>${q1_24}='sim'</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>selected(${q1_23}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
@@ -3015,12 +3007,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>q1_26</t>
+          <t>q1_24</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Q1.26. Há eventos sazonais que afetam a escola/comunidade (safras, secas, chuvas, festas, etc.)?</t>
+          <t>Q1.24. Essas atividades têm impacto percebido no ambiente ou na comunidade?</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -3039,19 +3031,19 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>q1_27</t>
+          <t>q1_25</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Q1.27. Qual é esse evento? Descreva-o.</t>
+          <t>Q1.25. Descreva os impactos percebidos por atividade</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>${q1_26}='sim'</t>
+          <t>${q1_24}='sim'</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -3066,26 +3058,22 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>select_multiple meses</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>q1_28</t>
+          <t>q1_26</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Q1.28. Em quais meses ele costuma ocorrer?</t>
+          <t>Q1.26. Há eventos sazonais que afetam a escola/comunidade (safras, secas, chuvas, festas, etc.)?</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>${q1_26}='sim'</t>
-        </is>
-      </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
@@ -3099,12 +3087,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>q1_29</t>
+          <t>q1_27</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Q1.29. Qual o impacto desse evento na escola?</t>
+          <t>Q1.27. Qual é esse evento? Descreva-o.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -3126,26 +3114,26 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>select_multiple meses</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>q1_30</t>
+          <t>q1_28</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Q1.30. Há histórico de eventos climáticos extremos que afetaram a escola/comunidade?</t>
+          <t>Q1.28. Em quais meses ele costuma ocorrer?</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>${q1_26}='sim'</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
@@ -3159,19 +3147,19 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>q1_31</t>
+          <t>q1_29</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Q1.31. Descreva o(s) evento(s)</t>
+          <t>Q1.29. Qual o impacto desse evento na escola?</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>${q1_30}='sim'</t>
+          <t>${q1_26}='sim'</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -3186,26 +3174,26 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>q1_32</t>
+          <t>q1_30</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Q1.32. Quando ocorreu(ram)?</t>
+          <t>Q1.30. Há histórico de eventos climáticos extremos que afetaram a escola/comunidade?</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>${q1_30}='sim'</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
@@ -3214,17 +3202,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>select_multiple impacto_clima</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>q1_33</t>
+          <t>q1_31</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Q1.33. Impactos observados</t>
+          <t>Q1.31. Descreva o(s) evento(s)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
@@ -3234,7 +3222,11 @@
           <t>${q1_30}='sim'</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
@@ -3247,19 +3239,19 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>q1_33_outro</t>
+          <t>q1_32</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q1.32. Quando ocorreu(ram)?</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
+          <t>${q1_30}='sim'</t>
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
@@ -3270,17 +3262,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_clima</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>q1_34</t>
+          <t>q1_33</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Q1.34. O que a escola/comunidade aprendeu com esse evento?</t>
+          <t>Q1.33. Impactos observados</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
@@ -3290,11 +3282,7 @@
           <t>${q1_30}='sim'</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
@@ -3307,26 +3295,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>q1_35</t>
+          <t>q1_33_outro</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Q1.35. Quais são as características-chave deste território, na sua leitura?</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Pense, por exemplo, em: relação com a água (rios, córregos, abastecimento), vegetação e áreas verdes, uso do solo predominante, memória e cultura local, riscos já percebidos e atividades econômicas mais presentes.</t>
-        </is>
-      </c>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
@@ -3339,21 +3323,21 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>q1_36</t>
+          <t>q1_34</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Q1.36. Há algum aspecto do território que vocês reconhecem não saber ainda?</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>'Não sabemos' é uma resposta válida — isso vira uma lacuna de conhecimento registrada.</t>
-        </is>
-      </c>
+          <t>Q1.34. O que a escola/comunidade aprendeu com esse evento?</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>${q1_30}='sim'</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr">
         <is>
           <t>multiline</t>
@@ -3366,23 +3350,31 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>evid_e1</t>
+          <t>q1_35</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Evidências — Evidências sobre a escola e o território</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>Q1.35. Quais são as características-chave deste território, na sua leitura?</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Pense, por exemplo, em: relação com a água (rios, córregos, abastecimento), vegetação e áreas verdes, uso do solo predominante, memória e cultura local, riscos já percebidos e atividades econômicas mais presentes.</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr"/>
@@ -3390,23 +3382,31 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>evid_e1_nota</t>
+          <t>q1_36</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>Q1.36. Há algum aspecto do território que vocês reconhecem não saber ainda?</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>'Não sabemos' é uma resposta válida — isso vira uma lacuna de conhecimento registrada.</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr"/>
@@ -3414,17 +3414,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>select_one tipo_evid</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>evid_e1_tipo</t>
+          <t>evid_e1</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Tipo de evidência</t>
+          <t>Evidências — Evidências sobre a escola e o território</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
@@ -3438,26 +3438,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>evid_e1_tipo_outro</t>
+          <t>evid_e1_nota</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>${evid_e1_tipo}='outro'</t>
-        </is>
-      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr"/>
@@ -3466,27 +3462,23 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one tipo_evid</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>evid_e1_desc</t>
+          <t>evid_e1_tipo</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Descreva a evidência</t>
+          <t>Tipo de evidência</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr"/>
@@ -3494,22 +3486,26 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>evid_e1_anexo</t>
+          <t>evid_e1_tipo_outro</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Anexo (foto/documento) — opcional</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>${evid_e1_tipo}='outro'</t>
+        </is>
+      </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
@@ -3518,15 +3514,27 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>evid_e1_desc</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Descreva a evidência</t>
+        </is>
+      </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
@@ -3534,11 +3542,19 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
+          <t>file</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>evid_e1_anexo</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Anexo (foto/documento) — opcional</t>
+        </is>
+      </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -3546,6 +3562,38 @@
       <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>